<commit_message>
Update output Excel files and add hollywood.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/home.xlsx
+++ b/output/home.xlsx
@@ -418,14 +418,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
     <col width="47" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
@@ -488,7 +488,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Peddi.jpg</t>
+          <t>home/06-06-2026/Peddi.jpg</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Ugly Story.jpg</t>
+          <t>home/06-06-2026/Ugly Story.jpg</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -558,24 +558,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>home/06-05-2026/29.jpg</t>
+          <t>home/06-06-2026/29.jpg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=qWSGdwHeKD4</t>
+          <t>https://www.youtube.com/watch?v=BwnSbiNMe60</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>KD: The Devil</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -593,24 +593,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Patriot.jpg</t>
+          <t>home/06-06-2026/KD The Devil.jpg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+          <t>https://www.youtube.com/watch?v=yQLKrS5N4KU</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KD: The Devil</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -628,24 +628,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>home/06-05-2026/KD The Devil.jpg</t>
+          <t>home/06-06-2026/Patriot.jpg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=yQLKrS5N4KU</t>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>The Rise of Ashoka</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -663,24 +663,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Patriot.jpg</t>
+          <t>home/06-06-2026/The Rise of Ashoka.jpg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Peter</t>
+          <t>Godari Gattupaina</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -698,24 +698,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Peter.jpg</t>
+          <t>home/06-06-2026/Godari Gattupaina.jpg</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=T7vWnJ8yuQs</t>
+          <t>https://www.youtube.com/watch?v=Q2ea_B_Y67M</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The Rise of Ashoka</t>
+          <t>Trikala: Script of God</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -733,24 +733,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>home/06-05-2026/The Rise of Ashoka.jpg</t>
+          <t>home/06-06-2026/Trikala Script of God.jpg</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+          <t>https://www.youtube.com/watch?v=U098Oyg8nYo</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -768,24 +768,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>home/06-05-2026/29.jpg</t>
+          <t>home/06-06-2026/Patriot.jpg</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=qWSGdwHeKD4</t>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>Sukhamano Sukhamann</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -803,24 +803,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Patriot.jpg</t>
+          <t>home/06-06-2026/Sukhamano Sukhamann.jpg</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+          <t>https://www.youtube.com/watch?v=YiYDvpWNK3o</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ugly Story</t>
+          <t>Carmeni Selvam</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -838,24 +838,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Ugly Story.jpg</t>
+          <t>home/06-06-2026/Carmeni Selvam.jpg</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+          <t>https://www.youtube.com/watch?v=W4BLjlRo4Bs</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>The Rise of Ashoka</t>
+          <t>Blast Zone</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -873,24 +873,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>home/06-05-2026/The Rise of Ashoka.jpg</t>
+          <t>home/06-06-2026/Blast Zone.jpg</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+          <t>https://www.youtube.com/watch?v=_vbRwxitX2o</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Office Romance</t>
+          <t>Maa Behen</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -908,24 +908,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Office Romance.jpg</t>
+          <t>home/06-06-2026/Maa Behen.jpg</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=M7KrcId8LQg</t>
+          <t>https://www.youtube.com/watch?v=xYbLpsEhcfA</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>The Marked Woman</t>
+          <t>Kattalan</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -943,24 +943,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>home/06-05-2026/The Marked Woman.jpg</t>
+          <t>home/06-06-2026/Kattalan.jpg</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=161b4xLkokE</t>
+          <t>https://www.youtube.com/watch?v=iQMvxXmCk9I</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ugly Story</t>
+          <t>Ramani Kalyanam</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -978,34 +978,34 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Ugly Story.jpg</t>
+          <t>home/06-06-2026/Ramani Kalyanam.jpg</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+          <t>https://www.youtube.com/watch?v=Iax6gOtJSw4</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sukhamano Sukhamann</t>
+          <t>Beast of War</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1013,24 +1013,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Sukhamano Sukhamann.jpg</t>
+          <t>home/06-06-2026/Beast of War.jpg</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=YiYDvpWNK3o</t>
+          <t>https://www.youtube.com/watch?v=x4Dk6joTDRg</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>The Rise of Ashoka</t>
+          <t>Sandigdham</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1048,24 +1048,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>home/06-05-2026/The Rise of Ashoka.jpg</t>
+          <t>home/06-06-2026/Sandigdham.jpg</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+          <t>https://www.youtube.com/watch?v=wTYXAINrYkw</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ugly Story</t>
+          <t>Kara</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1083,24 +1083,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>home/06-05-2026/Ugly Story.jpg</t>
+          <t>home/06-06-2026/Kara.jpg</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+          <t>https://www.youtube.com/watch?v=xkQS_TET5NI</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Maa Behen</t>
+          <t>KD: The Devil</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Kannada</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1118,24 +1118,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>home/06-04-2026/Maa Behen.jpg</t>
+          <t>home/06-06-2026/KD The Devil.jpg</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xYbLpsEhcfA</t>
+          <t>https://www.youtube.com/watch?v=yQLKrS5N4KU</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Momacu</t>
+          <t>Purushaha</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1153,24 +1153,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>home/06-04-2026/Momacu.jpg</t>
+          <t>home/06-06-2026/Purushaha.jpg</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ebWqjLUBgqE</t>
+          <t>https://www.youtube.com/watch?v=xs_NcJrsVy8</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Maa Behen</t>
+          <t>Hai Jawani Toh Ishq Hona Hai</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1188,34 +1188,34 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>home/06-04-2026/Maa Behen.jpg</t>
+          <t>home/06-06-2026/Hai Jawani Toh Ishq Hona Hai.jpg</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xYbLpsEhcfA</t>
+          <t>https://www.youtube.com/watch?v=rFOdIv1jwhc</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Premam Madhuram</t>
+          <t>Summer House</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1223,34 +1223,34 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>home/06-04-2026/Premam Madhuram.jpg</t>
+          <t>home/06-06-2026/Summer House.jpg</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=RkMt3-2m2mw</t>
+          <t>https://www.youtube.com/watch?v=9wGlGOhyLZk</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Beast of War</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1258,24 +1258,24 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>home/06-04-2026/Beast of War.jpg</t>
+          <t>home/06-06-2026/Patriot.jpg</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=x4Dk6joTDRg</t>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Godari Gattupaina</t>
+          <t>Juniors Journey</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1293,19 +1293,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Godari Gattupaina.jpg</t>
+          <t>home/06-06-2026/Juniors Journey.jpg</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uWgcpFbSnz8</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Blast Zone</t>
+          <t>Ginny Weds Sunny 2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1315,7 +1320,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1323,19 +1328,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Blast Zone.jpg</t>
+          <t>home/06-06-2026/Ginny Weds Sunny 2.jpg</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=NO7OOWCWmM0</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Carmeni Selvam</t>
+          <t>Peter</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1345,7 +1355,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Kannada</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1353,19 +1363,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Carmeni Selvam.jpg</t>
+          <t>home/06-06-2026/Peter.jpg</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=y25zcSqAdVs</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kattalan</t>
+          <t>The Rise of Ashoka</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1375,7 +1390,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1383,19 +1398,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Kattalan.jpg</t>
+          <t>home/06-06-2026/The Rise of Ashoka.jpg</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Kara</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1405,7 +1425,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1413,19 +1433,24 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Kara.jpg</t>
+          <t>home/06-06-2026/29.jpg</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BwnSbiNMe60</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sandigdham</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1435,7 +1460,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1443,19 +1468,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Sandigdham.jpg</t>
+          <t>home/06-06-2026/Patriot.jpg</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Purushaha</t>
+          <t>Ugly Story</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1465,7 +1495,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1473,19 +1503,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Purushaha.jpg</t>
+          <t>home/06-06-2026/Ugly Story.jpg</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ramani Kalyanam</t>
+          <t>The Rise of Ashoka</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1495,7 +1530,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Kannada</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1503,19 +1538,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Ramani Kalyanam.jpg</t>
+          <t>home/06-06-2026/The Rise of Ashoka.jpg</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bhishmar</t>
+          <t>Office Romance</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1525,7 +1565,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1533,462 +1573,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>home/06-02-2026/Bhishmar.jpg</t>
+          <t>home/06-06-2026/Office Romance.jpg</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M7KrcId8LQg</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Madhuvidhu</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Malayalam</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Madhuvidhu.jpg</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Telugu</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/14.jpg</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Lee Cronin’s The Mummy</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Lee Cronin’s The Mummy.jpg</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Carmeni Selvam</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Telugu</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Carmeni Selvam.jpg</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Rescue Dawn</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>2006</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Rescue Dawn.jpg</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Aaahladam</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Malayalam</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Aaahladam.jpg</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Trikala: Script of God</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Telugu</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Trikala Script of God.jpg</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Blast Zone</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Telugu</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Blast Zone.jpg</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Kattalan</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Telugu</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Kattalan.jpg</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Sandigdham</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Telugu</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Sandigdham.jpg</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>The Exorcism Of Emily Rose</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>2005</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/The Exorcism Of Emily Rose.jpg</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Kattalan</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Hindi</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Kattalan.jpg</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Purushaha</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Telugu</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Purushaha.jpg</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Faces</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Faces.jpg</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Nawab Cafe</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>home/06-02-2026/Nawab Cafe.jpg</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -2003,7 +1598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2025,31 +1620,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update home.xlsx output file
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/home.xlsx
+++ b/output/home.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Peddi</t>
+          <t>Sing Geetham</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -488,24 +488,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Peddi.jpg</t>
+          <t>home/06-16-2026/Sing Geetham.jpg</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=sF2dj7ycZvA</t>
+          <t>https://www.youtube.com/watch?v=8CzkA3WXjtQ</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ugly Story</t>
+          <t>Kenatha Kanom</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -523,24 +523,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Ugly Story.jpg</t>
+          <t>home/06-16-2026/Kenatha Kanom.jpg</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+          <t>https://www.youtube.com/watch?v=-qogxgbsxOQ</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>Veerabhadrudu</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -558,24 +558,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>home/06-06-2026/29.jpg</t>
+          <t>home/06-16-2026/Veerabhadrudu.jpg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=BwnSbiNMe60</t>
+          <t>https://www.youtube.com/watch?v=vH0Q5t_JUng</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KD: The Devil</t>
+          <t>Dridam</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -593,24 +593,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>home/06-06-2026/KD The Devil.jpg</t>
+          <t>home/06-16-2026/Dridam.jpg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=yQLKrS5N4KU</t>
+          <t>https://www.youtube.com/watch?v=AiFCD2aSnlc</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>Sattendru Maarudhu Vaanilai</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -628,24 +628,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Patriot.jpg</t>
+          <t>home/06-16-2026/Sattendru Maarudhu Vaanilai.jpg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+          <t>https://www.youtube.com/watch?v=Lbxw9Q3YmMw</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The Rise of Ashoka</t>
+          <t>Dridam</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -663,34 +663,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>home/06-06-2026/The Rise of Ashoka.jpg</t>
+          <t>home/06-16-2026/Dridam.jpg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+          <t>https://www.youtube.com/watch?v=AiFCD2aSnlc</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Godari Gattupaina</t>
+          <t>Pongala</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -698,24 +698,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Godari Gattupaina.jpg</t>
+          <t>home/06-16-2026/Pongala.jpg</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Q2ea_B_Y67M</t>
+          <t>https://www.youtube.com/watch?v=CDjL0lbpr40</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Trikala: Script of God</t>
+          <t>Shelter</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -733,24 +733,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Trikala Script of God.jpg</t>
+          <t>home/06-16-2026/Shelter.jpg</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=U098Oyg8nYo</t>
+          <t>https://www.youtube.com/watch?v=whOG1iwBGnM</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>Whistle</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -768,24 +768,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Patriot.jpg</t>
+          <t>home/06-16-2026/Whistle.jpg</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+          <t>https://www.youtube.com/watch?v=a6gxDFGte5M</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sukhamano Sukhamann</t>
+          <t>Kenatha Kanom</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -803,24 +803,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Sukhamano Sukhamann.jpg</t>
+          <t>home/06-16-2026/Kenatha Kanom.jpg</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=YiYDvpWNK3o</t>
+          <t>https://www.youtube.com/watch?v=-qogxgbsxOQ</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Carmeni Selvam</t>
+          <t>Kenatha Kanom</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -838,34 +838,34 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Carmeni Selvam.jpg</t>
+          <t>home/06-16-2026/Kenatha Kanom.jpg</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=W4BLjlRo4Bs</t>
+          <t>https://www.youtube.com/watch?v=-qogxgbsxOQ</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Blast Zone</t>
+          <t>The Deep</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -873,34 +873,34 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Blast Zone.jpg</t>
+          <t>home/06-16-2026/The Deep.jpg</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=_vbRwxitX2o</t>
+          <t>https://www.youtube.com/watch?v=qqdagoaQM7w</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Maa Behen</t>
+          <t>Seven Years in Tibet</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -908,24 +908,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Maa Behen.jpg</t>
+          <t>home/06-16-2026/Seven Years in Tibet.jpg</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xYbLpsEhcfA</t>
+          <t>https://www.youtube.com/watch?v=m9a_7WFcPlI</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kattalan</t>
+          <t>Kolahalamedu</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -943,24 +943,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Kattalan.jpg</t>
+          <t>home/06-16-2026/Kolahalamedu.jpg</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=iQMvxXmCk9I</t>
+          <t>https://www.youtube.com/watch?v=431lKAQyxd0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ramani Kalyanam</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Telugu Dubbed</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -978,34 +978,34 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Ramani Kalyanam.jpg</t>
+          <t>home/06-16-2026/Normal.jpg</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Iax6gOtJSw4</t>
+          <t>https://www.youtube.com/watch?v=aGdWT9_cEQY</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Beast of War</t>
+          <t>Sing Geetham</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Telugu Dubbed</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1013,24 +1013,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Beast of War.jpg</t>
+          <t>home/06-16-2026/Sing Geetham.jpg</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=x4Dk6joTDRg</t>
+          <t>https://www.youtube.com/watch?v=8CzkA3WXjtQ</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sandigdham</t>
+          <t>Vikalpa</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Kannada</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1048,24 +1048,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Sandigdham.jpg</t>
+          <t>home/06-16-2026/Vikalpa.jpg</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=wTYXAINrYkw</t>
+          <t>https://www.youtube.com/watch?v=9Jysx8EdZKM</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Kara</t>
+          <t>Dridam</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1083,24 +1083,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Kara.jpg</t>
+          <t>home/06-16-2026/Dridam.jpg</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xkQS_TET5NI</t>
+          <t>https://www.youtube.com/watch?v=AiFCD2aSnlc</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>KD: The Devil</t>
+          <t>Karuppu</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1118,24 +1118,24 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>home/06-06-2026/KD The Devil.jpg</t>
+          <t>home/06-16-2026/Karuppu.jpg</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=yQLKrS5N4KU</t>
+          <t>https://www.youtube.com/watch?v=JpVl_-1YgIo</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Purushaha</t>
+          <t>Sshhh Season 3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1153,24 +1153,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Purushaha.jpg</t>
+          <t>home/06-16-2026/Sshhh Season 3.jpg</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xs_NcJrsVy8</t>
+          <t>https://www.youtube.com/watch?v=92eqbag5gRU</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hai Jawani Toh Ishq Hona Hai</t>
+          <t>R.L. Stine’s Pumpkinhead</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Telugu Dubbed</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1188,24 +1188,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Hai Jawani Toh Ishq Hona Hai.jpg</t>
+          <t>home/06-16-2026/R.L. Stine’s Pumpkinhead.jpg</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=rFOdIv1jwhc</t>
+          <t>https://www.youtube.com/watch?v=gqmrfVrPJlY</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Summer House</t>
+          <t>Peddi</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Telugu Dubbed</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Summer House.jpg</t>
+          <t>home/06-06-2026/Peddi.jpg</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=9wGlGOhyLZk</t>
+          <t>https://www.youtube.com/watch?v=sF2dj7ycZvA</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1240,7 +1240,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>Ugly Story</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1258,12 +1258,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Patriot.jpg</t>
+          <t>home/06-06-2026/Ugly Story.jpg</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1275,7 +1275,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Juniors Journey</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Juniors Journey.jpg</t>
+          <t>home/06-06-2026/29.jpg</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=uWgcpFbSnz8</t>
+          <t>https://www.youtube.com/watch?v=BwnSbiNMe60</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1310,7 +1310,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ginny Weds Sunny 2</t>
+          <t>KD: The Devil</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1328,12 +1328,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Ginny Weds Sunny 2.jpg</t>
+          <t>home/06-06-2026/KD The Devil.jpg</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=NO7OOWCWmM0</t>
+          <t>https://www.youtube.com/watch?v=yQLKrS5N4KU</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1345,7 +1345,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Peter</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1363,12 +1363,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Peter.jpg</t>
+          <t>home/06-06-2026/Patriot.jpg</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=y25zcSqAdVs</t>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1415,7 +1415,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>Godari Gattupaina</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1433,12 +1433,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>home/06-06-2026/29.jpg</t>
+          <t>home/06-06-2026/Godari Gattupaina.jpg</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=BwnSbiNMe60</t>
+          <t>https://www.youtube.com/watch?v=Q2ea_B_Y67M</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1450,7 +1450,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>Trikala: Script of God</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Patriot.jpg</t>
+          <t>home/06-06-2026/Trikala Script of God.jpg</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+          <t>https://www.youtube.com/watch?v=U098Oyg8nYo</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1485,7 +1485,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ugly Story</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1503,12 +1503,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>home/06-06-2026/Ugly Story.jpg</t>
+          <t>home/06-06-2026/Patriot.jpg</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1520,7 +1520,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>The Rise of Ashoka</t>
+          <t>Sukhamano Sukhamann</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>home/06-06-2026/The Rise of Ashoka.jpg</t>
+          <t>home/06-06-2026/Sukhamano Sukhamann.jpg</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+          <t>https://www.youtube.com/watch?v=YiYDvpWNK3o</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1555,33 +1555,768 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Carmeni Selvam</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Carmeni Selvam.jpg</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=W4BLjlRo4Bs</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Blast Zone</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Blast Zone.jpg</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_vbRwxitX2o</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Maa Behen</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Maa Behen.jpg</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xYbLpsEhcfA</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Kattalan</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Kattalan.jpg</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iQMvxXmCk9I</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Ramani Kalyanam</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Telugu Dubbed</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Ramani Kalyanam.jpg</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Iax6gOtJSw4</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Beast of War</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Telugu Dubbed</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Beast of War.jpg</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=x4Dk6joTDRg</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sandigdham</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Sandigdham.jpg</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wTYXAINrYkw</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Kara</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Kara.jpg</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xkQS_TET5NI</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KD: The Devil</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Kannada</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/KD The Devil.jpg</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yQLKrS5N4KU</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Purushaha</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Purushaha.jpg</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xs_NcJrsVy8</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Hai Jawani Toh Ishq Hona Hai</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Hai Jawani Toh Ishq Hona Hai.jpg</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rFOdIv1jwhc</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Summer House</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Telugu Dubbed</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Summer House.jpg</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9wGlGOhyLZk</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Patriot</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Patriot.jpg</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Juniors Journey</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Malayalam</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Juniors Journey.jpg</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uWgcpFbSnz8</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Ginny Weds Sunny 2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Ginny Weds Sunny 2.jpg</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=NO7OOWCWmM0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Peter</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Kannada</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Peter.jpg</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=y25zcSqAdVs</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>The Rise of Ashoka</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/The Rise of Ashoka.jpg</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/29.jpg</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BwnSbiNMe60</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Patriot</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Patriot.jpg</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XTc2dLAgABI</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Ugly Story</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/Ugly Story.jpg</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>The Rise of Ashoka</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Kannada</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>home/06-06-2026/The Rise of Ashoka.jpg</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>Office Romance</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
         <is>
           <t>Telugu Dubbed</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>home/06-06-2026/Office Romance.jpg</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=M7KrcId8LQg</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>2026-06-06</t>
         </is>
@@ -1598,7 +2333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1620,10 +2355,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>32</v>
       </c>
     </row>

</xml_diff>